<commit_message>
dwh_gold: godkendte beskrivelser i TMDL og opstrømskilder i kataloget
- 70 godkendte beskrivelser skrevet tilbage som ///-linjer i fem
  tabelfiler. Ingen DAX, M eller egenskaber er ændret.
- catalog.xlsx: "Opstrøms kilde" udfyldt for alle tabeller og kolonner
  (bronze → silver → gold) ud fra gold.load_gold() og silver.load_silver()
  i supabase/migrations.
- Kataloget er genereret igen. Alle 82 beskrivelser er nu fra modellen
  eller godkendt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013At67Gwi9xCc2C5qN1Bh34
</commit_message>
<xml_diff>
--- a/output/dwh_gold/docs/catalog.xlsx
+++ b/output/dwh_gold/docs/catalog.xlsx
@@ -489,7 +489,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-29 19:56</t>
+          <t>2026-10-29 20:00</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -608,7 +608,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16">
@@ -697,7 +697,7 @@
     <col width="60" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="45" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="19" customWidth="1" min="17" max="17"/>
   </cols>
@@ -828,7 +828,11 @@
       </c>
       <c r="M2" s="4" t="inlineStr"/>
       <c r="N2" s="4" t="inlineStr"/>
-      <c r="O2" s="4" t="inlineStr"/>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>Ingen – measure-tabel i Power BI</t>
+        </is>
+      </c>
       <c r="P2" s="4" t="inlineStr">
         <is>
           <t>Fra model</t>
@@ -891,10 +895,14 @@
       </c>
       <c r="M3" s="4" t="inlineStr"/>
       <c r="N3" s="4" t="inlineStr"/>
-      <c r="O3" s="4" t="inlineStr"/>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>gold.load_gold(): silver.crm_cust_info (CRM) + silver.erp_cust_az12 og silver.erp_loc_a101 (ERP, left join på cst_key = cid) ← bronze</t>
+        </is>
+      </c>
       <c r="P3" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -954,7 +962,11 @@
       </c>
       <c r="M4" s="4" t="inlineStr"/>
       <c r="N4" s="4" t="inlineStr"/>
-      <c r="O4" s="4" t="inlineStr"/>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query ud fra datoerne i fact_sales (ingen tabel i Supabase)</t>
+        </is>
+      </c>
       <c r="P4" s="4" t="inlineStr">
         <is>
           <t>Fra model</t>
@@ -1021,10 +1033,14 @@
       </c>
       <c r="M5" s="4" t="inlineStr"/>
       <c r="N5" s="4" t="inlineStr"/>
-      <c r="O5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>gold.load_gold(): silver.crm_prd_info (CRM) + silver.erp_px_cat_g1v2 (ERP, left join på cat_id = id), kun aktuelle produkter (prd_end_dt is null) ← bronze</t>
+        </is>
+      </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1088,10 +1104,14 @@
       </c>
       <c r="M6" s="4" t="inlineStr"/>
       <c r="N6" s="4" t="inlineStr"/>
-      <c r="O6" s="4" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>gold.load_gold(): silver.crm_sales_details (CRM) + opslag i gold.dim_products og gold.dim_customers ← bronze.crm_sales_details</t>
+        </is>
+      </c>
       <c r="P6" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1139,7 +1159,7 @@
     <col width="60" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="45" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
   </cols>
@@ -1320,10 +1340,14 @@
       </c>
       <c r="R2" s="4" t="inlineStr"/>
       <c r="S2" s="4" t="inlineStr"/>
-      <c r="T2" s="4" t="inlineStr"/>
+      <c r="T2" s="4" t="inlineStr">
+        <is>
+          <t>Surrogatnøgle i gold: row_number() over cst_id</t>
+        </is>
+      </c>
       <c r="U2" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
@@ -1392,10 +1416,14 @@
       </c>
       <c r="R3" s="4" t="inlineStr"/>
       <c r="S3" s="4" t="inlineStr"/>
-      <c r="T3" s="4" t="inlineStr"/>
+      <c r="T3" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_id ← bronze.crm_cust_info (nyeste række pr. kunde)</t>
+        </is>
+      </c>
       <c r="U3" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
@@ -1456,10 +1484,14 @@
       </c>
       <c r="R4" s="4" t="inlineStr"/>
       <c r="S4" s="4" t="inlineStr"/>
-      <c r="T4" s="4" t="inlineStr"/>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_key ← bronze.crm_cust_info</t>
+        </is>
+      </c>
       <c r="U4" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
@@ -1528,10 +1560,14 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T5" s="4" t="inlineStr"/>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_firstname (trimmet) ← bronze.crm_cust_info</t>
+        </is>
+      </c>
       <c r="U5" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
@@ -1600,10 +1636,14 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr"/>
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_lastname (trimmet) ← bronze.crm_cust_info</t>
+        </is>
+      </c>
       <c r="U6" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V6" t="inlineStr">
@@ -1668,10 +1708,14 @@
       </c>
       <c r="R7" s="4" t="inlineStr"/>
       <c r="S7" s="4" t="inlineStr"/>
-      <c r="T7" s="4" t="inlineStr"/>
+      <c r="T7" s="4" t="inlineStr">
+        <is>
+          <t>silver.erp_loc_a101.cntry (DE→Germany, US/USA→United States, tom→n/a) ← bronze.erp_loc_a101</t>
+        </is>
+      </c>
       <c r="U7" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V7" t="inlineStr">
@@ -1732,10 +1776,14 @@
       </c>
       <c r="R8" s="4" t="inlineStr"/>
       <c r="S8" s="4" t="inlineStr"/>
-      <c r="T8" s="4" t="inlineStr"/>
+      <c r="T8" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_marital_status (S/M→Single/Married) ← bronze.crm_cust_info</t>
+        </is>
+      </c>
       <c r="U8" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -1804,10 +1852,14 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T9" s="4" t="inlineStr"/>
+      <c r="T9" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_gndr; hvis n/a: silver.erp_cust_az12.gen ← bronze (CRM primær, ERP fallback)</t>
+        </is>
+      </c>
       <c r="U9" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
@@ -1880,10 +1932,14 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T10" s="4" t="inlineStr"/>
+      <c r="T10" s="4" t="inlineStr">
+        <is>
+          <t>silver.erp_cust_az12.bdate (fremtidige datoer→NULL) ← bronze.erp_cust_az12</t>
+        </is>
+      </c>
       <c r="U10" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
@@ -1948,10 +2004,14 @@
       </c>
       <c r="R11" s="4" t="inlineStr"/>
       <c r="S11" s="4" t="inlineStr"/>
-      <c r="T11" s="4" t="inlineStr"/>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_create_date ← bronze.crm_cust_info</t>
+        </is>
+      </c>
       <c r="U11" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
@@ -2016,10 +2076,14 @@
       </c>
       <c r="R12" s="4" t="inlineStr"/>
       <c r="S12" s="4" t="inlineStr"/>
-      <c r="T12" s="4" t="inlineStr"/>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (ingen kilde i Supabase)</t>
+        </is>
+      </c>
       <c r="U12" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
@@ -2080,10 +2144,14 @@
       </c>
       <c r="R13" s="4" t="inlineStr"/>
       <c r="S13" s="4" t="inlineStr"/>
-      <c r="T13" s="4" t="inlineStr"/>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (ingen kilde i Supabase)</t>
+        </is>
+      </c>
       <c r="U13" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -2140,10 +2208,14 @@
       </c>
       <c r="R14" s="4" t="inlineStr"/>
       <c r="S14" s="4" t="inlineStr"/>
-      <c r="T14" s="4" t="inlineStr"/>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (ingen kilde i Supabase)</t>
+        </is>
+      </c>
       <c r="U14" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
@@ -2208,10 +2280,14 @@
       </c>
       <c r="R15" s="4" t="inlineStr"/>
       <c r="S15" s="4" t="inlineStr"/>
-      <c r="T15" s="4" t="inlineStr"/>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (ingen kilde i Supabase)</t>
+        </is>
+      </c>
       <c r="U15" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
@@ -2276,10 +2352,14 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T16" s="4" t="inlineStr"/>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (ingen kilde i Supabase)</t>
+        </is>
+      </c>
       <c r="U16" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
@@ -2336,10 +2416,14 @@
       </c>
       <c r="R17" s="4" t="inlineStr"/>
       <c r="S17" s="4" t="inlineStr"/>
-      <c r="T17" s="4" t="inlineStr"/>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (ingen kilde i Supabase)</t>
+        </is>
+      </c>
       <c r="U17" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
@@ -2408,10 +2492,14 @@
       </c>
       <c r="R18" s="4" t="inlineStr"/>
       <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (ingen kilde i Supabase)</t>
+        </is>
+      </c>
       <c r="U18" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
@@ -2472,10 +2560,14 @@
       </c>
       <c r="R19" s="4" t="inlineStr"/>
       <c r="S19" s="4" t="inlineStr"/>
-      <c r="T19" s="4" t="inlineStr"/>
+      <c r="T19" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (ingen kilde i Supabase)</t>
+        </is>
+      </c>
       <c r="U19" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
@@ -2540,10 +2632,14 @@
       </c>
       <c r="R20" s="4" t="inlineStr"/>
       <c r="S20" s="4" t="inlineStr"/>
-      <c r="T20" s="4" t="inlineStr"/>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (ingen kilde i Supabase)</t>
+        </is>
+      </c>
       <c r="U20" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
@@ -2608,10 +2704,14 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T21" s="4" t="inlineStr"/>
+      <c r="T21" s="4" t="inlineStr">
+        <is>
+          <t>Genereres i Power Query (ingen kilde i Supabase)</t>
+        </is>
+      </c>
       <c r="U21" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
@@ -2684,10 +2784,14 @@
       </c>
       <c r="R22" s="4" t="inlineStr"/>
       <c r="S22" s="4" t="inlineStr"/>
-      <c r="T22" s="4" t="inlineStr"/>
+      <c r="T22" s="4" t="inlineStr">
+        <is>
+          <t>Surrogatnøgle i gold: row_number() over prd_start_dt, prd_key</t>
+        </is>
+      </c>
       <c r="U22" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
@@ -2756,10 +2860,14 @@
       </c>
       <c r="R23" s="4" t="inlineStr"/>
       <c r="S23" s="4" t="inlineStr"/>
-      <c r="T23" s="4" t="inlineStr"/>
+      <c r="T23" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_id ← bronze.crm_prd_info</t>
+        </is>
+      </c>
       <c r="U23" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
@@ -2820,10 +2928,14 @@
       </c>
       <c r="R24" s="4" t="inlineStr"/>
       <c r="S24" s="4" t="inlineStr"/>
-      <c r="T24" s="4" t="inlineStr"/>
+      <c r="T24" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_key (prd_key fra tegn 7) ← bronze.crm_prd_info</t>
+        </is>
+      </c>
       <c r="U24" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -2900,10 +3012,14 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T25" s="4" t="inlineStr"/>
+      <c r="T25" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_nm ← bronze.crm_prd_info</t>
+        </is>
+      </c>
       <c r="U25" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
@@ -2968,10 +3084,14 @@
       </c>
       <c r="R26" s="4" t="inlineStr"/>
       <c r="S26" s="4" t="inlineStr"/>
-      <c r="T26" s="4" t="inlineStr"/>
+      <c r="T26" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.cat_id (første 5 tegn af prd_key, - → _) ← bronze.crm_prd_info</t>
+        </is>
+      </c>
       <c r="U26" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V26" t="inlineStr">
@@ -3040,10 +3160,14 @@
       </c>
       <c r="R27" s="4" t="inlineStr"/>
       <c r="S27" s="4" t="inlineStr"/>
-      <c r="T27" s="4" t="inlineStr"/>
+      <c r="T27" s="4" t="inlineStr">
+        <is>
+          <t>silver.erp_px_cat_g1v2.cat ← bronze.erp_px_cat_g1v2</t>
+        </is>
+      </c>
       <c r="U27" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V27" t="inlineStr">
@@ -3108,10 +3232,14 @@
       </c>
       <c r="R28" s="4" t="inlineStr"/>
       <c r="S28" s="4" t="inlineStr"/>
-      <c r="T28" s="4" t="inlineStr"/>
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t>silver.erp_px_cat_g1v2.subcat ← bronze.erp_px_cat_g1v2</t>
+        </is>
+      </c>
       <c r="U28" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V28" t="inlineStr">
@@ -3172,10 +3300,14 @@
       </c>
       <c r="R29" s="4" t="inlineStr"/>
       <c r="S29" s="4" t="inlineStr"/>
-      <c r="T29" s="4" t="inlineStr"/>
+      <c r="T29" s="4" t="inlineStr">
+        <is>
+          <t>silver.erp_px_cat_g1v2.maintenance ← bronze.erp_px_cat_g1v2</t>
+        </is>
+      </c>
       <c r="U29" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V29" t="inlineStr">
@@ -3244,10 +3376,14 @@
       </c>
       <c r="R30" s="4" t="inlineStr"/>
       <c r="S30" s="4" t="inlineStr"/>
-      <c r="T30" s="4" t="inlineStr"/>
+      <c r="T30" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_cost (NULL→0) ← bronze.crm_prd_info</t>
+        </is>
+      </c>
       <c r="U30" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V30" t="inlineStr">
@@ -3308,10 +3444,14 @@
       </c>
       <c r="R31" s="4" t="inlineStr"/>
       <c r="S31" s="4" t="inlineStr"/>
-      <c r="T31" s="4" t="inlineStr"/>
+      <c r="T31" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_line (M/R/S/T→Mountain/Road/Other Sales/Touring) ← bronze.crm_prd_info</t>
+        </is>
+      </c>
       <c r="U31" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V31" t="inlineStr">
@@ -3376,10 +3516,14 @@
       </c>
       <c r="R32" s="4" t="inlineStr"/>
       <c r="S32" s="4" t="inlineStr"/>
-      <c r="T32" s="4" t="inlineStr"/>
+      <c r="T32" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_start_dt ← bronze.crm_prd_info</t>
+        </is>
+      </c>
       <c r="U32" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V32" t="inlineStr">
@@ -3452,10 +3596,14 @@
       </c>
       <c r="R33" s="4" t="inlineStr"/>
       <c r="S33" s="4" t="inlineStr"/>
-      <c r="T33" s="4" t="inlineStr"/>
+      <c r="T33" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_ord_num ← bronze.crm_sales_details</t>
+        </is>
+      </c>
       <c r="U33" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V33" t="inlineStr">
@@ -3524,10 +3672,14 @@
       </c>
       <c r="R34" s="4" t="inlineStr"/>
       <c r="S34" s="4" t="inlineStr"/>
-      <c r="T34" s="4" t="inlineStr"/>
+      <c r="T34" s="4" t="inlineStr">
+        <is>
+          <t>gold.dim_products.product_key via sls_prd_key = product_number</t>
+        </is>
+      </c>
       <c r="U34" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V34" t="inlineStr">
@@ -3600,10 +3752,14 @@
       </c>
       <c r="R35" s="4" t="inlineStr"/>
       <c r="S35" s="4" t="inlineStr"/>
-      <c r="T35" s="4" t="inlineStr"/>
+      <c r="T35" s="4" t="inlineStr">
+        <is>
+          <t>gold.dim_customers.customer_key via sls_cust_id = customer_id</t>
+        </is>
+      </c>
       <c r="U35" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
@@ -3676,10 +3832,14 @@
       </c>
       <c r="R36" s="4" t="inlineStr"/>
       <c r="S36" s="4" t="inlineStr"/>
-      <c r="T36" s="4" t="inlineStr"/>
+      <c r="T36" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_order_dt (ugyldig yyyymmdd→NULL) ← bronze.crm_sales_details</t>
+        </is>
+      </c>
       <c r="U36" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V36" t="inlineStr">
@@ -3752,10 +3912,14 @@
           <t>Mulig PII - vurdér</t>
         </is>
       </c>
-      <c r="T37" s="4" t="inlineStr"/>
+      <c r="T37" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_ship_dt (ugyldig yyyymmdd→NULL) ← bronze.crm_sales_details</t>
+        </is>
+      </c>
       <c r="U37" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V37" t="inlineStr">
@@ -3820,10 +3984,14 @@
       </c>
       <c r="R38" s="4" t="inlineStr"/>
       <c r="S38" s="4" t="inlineStr"/>
-      <c r="T38" s="4" t="inlineStr"/>
+      <c r="T38" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_due_dt (ugyldig yyyymmdd→NULL) ← bronze.crm_sales_details</t>
+        </is>
+      </c>
       <c r="U38" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
@@ -3892,10 +4060,14 @@
       </c>
       <c r="R39" s="4" t="inlineStr"/>
       <c r="S39" s="4" t="inlineStr"/>
-      <c r="T39" s="4" t="inlineStr"/>
+      <c r="T39" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_sales (genberegnet som antal × |pris| hvis ugyldig) ← bronze.crm_sales_details</t>
+        </is>
+      </c>
       <c r="U39" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V39" t="inlineStr">
@@ -3964,10 +4136,14 @@
       </c>
       <c r="R40" s="4" t="inlineStr"/>
       <c r="S40" s="4" t="inlineStr"/>
-      <c r="T40" s="4" t="inlineStr"/>
+      <c r="T40" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_quantity ← bronze.crm_sales_details</t>
+        </is>
+      </c>
       <c r="U40" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V40" t="inlineStr">
@@ -4032,10 +4208,14 @@
       </c>
       <c r="R41" s="4" t="inlineStr"/>
       <c r="S41" s="4" t="inlineStr"/>
-      <c r="T41" s="4" t="inlineStr"/>
+      <c r="T41" s="4" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_price (salg/antal hvis ugyldig) ← bronze.crm_sales_details</t>
+        </is>
+      </c>
       <c r="U41" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="V41" t="inlineStr">
@@ -4343,7 +4523,7 @@
       <c r="R3" s="4" t="inlineStr"/>
       <c r="S3" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
@@ -4405,7 +4585,7 @@
       <c r="R4" s="4" t="inlineStr"/>
       <c r="S4" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -4471,7 +4651,7 @@
       <c r="R5" s="4" t="inlineStr"/>
       <c r="S5" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -4537,7 +4717,7 @@
       <c r="R6" s="4" t="inlineStr"/>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
@@ -4603,7 +4783,7 @@
       <c r="R7" s="4" t="inlineStr"/>
       <c r="S7" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
@@ -4747,7 +4927,7 @@
       <c r="R9" s="4" t="inlineStr"/>
       <c r="S9" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
@@ -4821,7 +5001,7 @@
       <c r="R10" s="4" t="inlineStr"/>
       <c r="S10" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
@@ -4895,7 +5075,7 @@
       <c r="R11" s="4" t="inlineStr"/>
       <c r="S11" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
@@ -4964,7 +5144,7 @@
       <c r="R12" s="4" t="inlineStr"/>
       <c r="S12" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
@@ -5032,7 +5212,7 @@
       <c r="R13" s="4" t="inlineStr"/>
       <c r="S13" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
@@ -5106,7 +5286,7 @@
       <c r="R14" s="4" t="inlineStr"/>
       <c r="S14" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
@@ -5175,7 +5355,7 @@
       <c r="R15" s="4" t="inlineStr"/>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
@@ -5321,7 +5501,7 @@
       <c r="R17" s="4" t="inlineStr"/>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
@@ -5692,7 +5872,7 @@
       <c r="R22" s="4" t="inlineStr"/>
       <c r="S22" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
@@ -5766,7 +5946,7 @@
       <c r="R23" s="4" t="inlineStr"/>
       <c r="S23" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
@@ -5930,7 +6110,7 @@
       <c r="R25" s="4" t="inlineStr"/>
       <c r="S25" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
@@ -6010,7 +6190,7 @@
       <c r="R26" s="4" t="inlineStr"/>
       <c r="S26" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
@@ -6083,7 +6263,7 @@
       <c r="R27" s="4" t="inlineStr"/>
       <c r="S27" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
@@ -6153,7 +6333,7 @@
       <c r="R28" s="4" t="inlineStr"/>
       <c r="S28" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T28" t="inlineStr">
@@ -6237,7 +6417,7 @@
       <c r="R29" s="4" t="inlineStr"/>
       <c r="S29" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T29" t="inlineStr">
@@ -6317,7 +6497,7 @@
       <c r="R30" s="4" t="inlineStr"/>
       <c r="S30" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
@@ -6390,7 +6570,7 @@
       <c r="R31" s="4" t="inlineStr"/>
       <c r="S31" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
@@ -6460,7 +6640,7 @@
       <c r="R32" s="4" t="inlineStr"/>
       <c r="S32" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
@@ -6544,7 +6724,7 @@
       <c r="R33" s="4" t="inlineStr"/>
       <c r="S33" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
@@ -6624,7 +6804,7 @@
       <c r="R34" s="4" t="inlineStr"/>
       <c r="S34" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
@@ -6697,7 +6877,7 @@
       <c r="R35" s="4" t="inlineStr"/>
       <c r="S35" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
@@ -6767,7 +6947,7 @@
       <c r="R36" s="4" t="inlineStr"/>
       <c r="S36" s="4" t="inlineStr">
         <is>
-          <t>AI-forslag</t>
+          <t>Godkendt</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">

</xml_diff>

<commit_message>
Kataloger genereret igen med strammere PII-tjek
Med claude-powerbi-skills PR #3 matcher PII-tjekket hele ord og tager
højde for tabellen:
- dwh_gold: 5 markeringer (fornavn, efternavn, civilstand, køn,
  fødselsdato). De falske alarmer month_name, day_name, product_name og
  shipping_date er væk.
- sales_model: 6 markeringer (customer_name, account_manager, street,
  city, primary_contact, user_email). De falske alarmer på navne for ting
  er væk.
"Mulig PII" viser grunden, og gamle auto-markeringer i Følsomhed er
ryddet. Beskrivelser, status og Opstrøms kilde er uændrede.
lineage.md og lineage.azdo.md er kun genereret igen (ny dato).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013At67Gwi9xCc2C5qN1Bh34
</commit_message>
<xml_diff>
--- a/output/dwh_gold/docs/catalog.xlsx
+++ b/output/dwh_gold/docs/catalog.xlsx
@@ -489,7 +489,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-29 20:00</t>
+          <t>2026-10-29 20:32</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="38" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
     <col width="60" customWidth="1" min="12" max="12"/>
@@ -1527,7 +1527,7 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja (firstname)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1603,7 +1603,7 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja (lastname)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1749,7 +1749,11 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Ja (marital)</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>gold.dim_customers.marital_status</t>
@@ -1775,7 +1779,11 @@
         </is>
       </c>
       <c r="R8" s="4" t="inlineStr"/>
-      <c r="S8" s="4" t="inlineStr"/>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>Mulig PII - vurdér</t>
+        </is>
+      </c>
       <c r="T8" s="4" t="inlineStr">
         <is>
           <t>silver.crm_cust_info.cst_marital_status (S/M→Single/Married) ← bronze.crm_cust_info</t>
@@ -1819,7 +1827,7 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja (gender)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1899,7 +1907,7 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja (birthdate)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2321,11 +2329,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
+      <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
           <t>Beregnet i dim_date (trin Maaned)</t>
@@ -2347,11 +2351,7 @@
         </is>
       </c>
       <c r="R16" s="4" t="inlineStr"/>
-      <c r="S16" s="4" t="inlineStr">
-        <is>
-          <t>Mulig PII - vurdér</t>
-        </is>
-      </c>
+      <c r="S16" s="4" t="inlineStr"/>
       <c r="T16" s="4" t="inlineStr">
         <is>
           <t>Genereres i Power Query (ingen kilde i Supabase)</t>
@@ -2673,11 +2673,7 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>Beregnet i dim_date (trin Ugedag)</t>
@@ -2699,11 +2695,7 @@
         </is>
       </c>
       <c r="R21" s="4" t="inlineStr"/>
-      <c r="S21" s="4" t="inlineStr">
-        <is>
-          <t>Mulig PII - vurdér</t>
-        </is>
-      </c>
+      <c r="S21" s="4" t="inlineStr"/>
       <c r="T21" s="4" t="inlineStr">
         <is>
           <t>Genereres i Power Query (ingen kilde i Supabase)</t>
@@ -2969,11 +2961,7 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
+      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>gold.dim_products.product_name</t>
@@ -3007,11 +2995,7 @@
         </is>
       </c>
       <c r="R25" s="4" t="inlineStr"/>
-      <c r="S25" s="4" t="inlineStr">
-        <is>
-          <t>Mulig PII - vurdér</t>
-        </is>
-      </c>
+      <c r="S25" s="4" t="inlineStr"/>
       <c r="T25" s="4" t="inlineStr">
         <is>
           <t>silver.crm_prd_info.prd_nm ← bronze.crm_prd_info</t>
@@ -3877,11 +3861,7 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
+      <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
           <t>gold.fact_sales.shipping_date</t>
@@ -3907,11 +3887,7 @@
         </is>
       </c>
       <c r="R37" s="4" t="inlineStr"/>
-      <c r="S37" s="4" t="inlineStr">
-        <is>
-          <t>Mulig PII - vurdér</t>
-        </is>
-      </c>
+      <c r="S37" s="4" t="inlineStr"/>
       <c r="T37" s="4" t="inlineStr">
         <is>
           <t>silver.crm_sales_details.sls_ship_dt (ugyldig yyyymmdd→NULL) ← bronze.crm_sales_details</t>

</xml_diff>

<commit_message>
Kataloger genereret igen med automatisk Opstrøms kilde
Begge kataloger er genereret igen med claude-powerbi-skills PR #5 (dwh_gold
med --sql supabase/migrations). Den nye kolonne "Opstrøms kilde (auto)"
viser den automatiske tekst ved siden af den håndskrevne. De håndskrevne
tekster i Opstrøms kilde er bevaret. Beskrivelser, status og TMDL er
uændrede.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013At67Gwi9xCc2C5qN1Bh34
</commit_message>
<xml_diff>
--- a/output/dwh_gold/docs/catalog.xlsx
+++ b/output/dwh_gold/docs/catalog.xlsx
@@ -16,8 +16,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kilder" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tabeller'!$A$1:$Q$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Kolonner'!$A$1:$V$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tabeller'!$A$1:$R$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Kolonner'!$A$1:$W$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Measures'!$A$1:$T$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dashboard'!$A$1:$G$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Relationer'!$A$1:$E$6</definedName>
@@ -489,7 +489,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-29 20:32</t>
+          <t>2026-10-29 20:58</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -697,9 +697,10 @@
     <col width="60" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="45" customWidth="1" min="15" max="15"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="19" customWidth="1" min="17" max="17"/>
+    <col width="45" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -786,6 +787,11 @@
       <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>Beskrivelseskilde</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Opstrøms kilde (auto)</t>
         </is>
       </c>
     </row>
@@ -843,6 +849,11 @@
           <t>TMDL</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Ingen – measure-tabel i Power BI</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -910,6 +921,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info, silver.erp_cust_az12, silver.erp_loc_a101 ← bronze.crm_cust_info, bronze.erp_cust_az12, bronze.erp_loc_a101</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -977,6 +993,11 @@
           <t>TMDL</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Genereret i Power Query ud fra fact_sales</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1048,6 +1069,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info, silver.erp_px_cat_g1v2 ← bronze.crm_prd_info, bronze.erp_px_cat_g1v2 (filter: pn.prd_end_dt is null)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1119,9 +1145,14 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>gold.dim_customers, gold.dim_products, silver.crm_sales_details ← bronze.crm_sales_details</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q6"/>
+  <autoFilter ref="A1:R6"/>
   <dataValidations count="1">
     <dataValidation sqref="P2:P6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Mangler,AI-forslag,Fra model,Redigeret,Godkendt"</formula1>
@@ -1137,7 +1168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:W41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1159,9 +1190,10 @@
     <col width="60" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="45" customWidth="1" min="20" max="20"/>
+    <col width="60" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="19" customWidth="1" min="22" max="22"/>
+    <col width="45" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1273,6 +1305,11 @@
       <c r="V1" s="2" t="inlineStr">
         <is>
           <t>Beskrivelseskilde</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>Opstrøms kilde (auto)</t>
         </is>
       </c>
     </row>
@@ -1355,6 +1392,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_id (afledt: row_number() over (order by ci.cst_id)) ← bronze.crm_cust_info.cst_id</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1429,6 +1471,11 @@
       <c r="V3" t="inlineStr">
         <is>
           <t>Excel</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_id ← bronze.crm_cust_info.cst_id</t>
         </is>
       </c>
     </row>
@@ -1499,6 +1546,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_key ← bronze.crm_cust_info.cst_key</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1575,6 +1627,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_firstname ← bronze.crm_cust_info.cst_firstname (afledt: trim(cst_firstname))</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1649,6 +1706,11 @@
       <c r="V6" t="inlineStr">
         <is>
           <t>Excel</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_lastname ← bronze.crm_cust_info.cst_lastname (afledt: trim(cst_lastname))</t>
         </is>
       </c>
     </row>
@@ -1723,6 +1785,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>silver.erp_loc_a101.cntry ← bronze.erp_loc_a101.cntry (afledt: case when trim(cntry) = 'DE' then 'Germany' when trim(cntry) in ('US', 'USA') t…)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1799,6 +1866,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_marital_status ← bronze.crm_cust_info.cst_marital_status (afledt: case when upper(trim(cst_marital_status)) = 'S' then 'Single' when upper(trim(c…)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1875,6 +1947,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_gndr + silver.erp_cust_az12.gen (afledt: case when ci.cst_gndr != 'n/a' then ci.cst_gndr else coalesce(ca.gen, 'n/a') end) ← bronze.crm_cust_info.cst_gndr + bronze.erp_cust_az12.gen (afledt: case when upper(trim(cst_gndr)) = 'F' then 'Female' when upper(trim(cst_gndr)) …; case when upper(trim(gen)) in ('F', 'FEMALE') then 'Female' when upper(trim(gen…)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1955,6 +2032,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>silver.erp_cust_az12.bdate ← bronze.erp_cust_az12.bdate (afledt: case when bdate &gt; now() then null else bdate end)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2027,6 +2109,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>silver.crm_cust_info.cst_create_date ← bronze.crm_cust_info.cst_create_date</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2099,6 +2186,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Genereret i Power Query (dim_date)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2165,6 +2257,11 @@
       <c r="V13" t="inlineStr">
         <is>
           <t>Excel</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query (dim_date): each Date.Year([date_key])</t>
         </is>
       </c>
     </row>
@@ -2231,6 +2328,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query (dim_date): each "K" &amp; Text.From(Date.QuarterOfYear([date_key]))</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2301,6 +2403,11 @@
       <c r="V15" t="inlineStr">
         <is>
           <t>Excel</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query (dim_date): each Date.Month([date_key])</t>
         </is>
       </c>
     </row>
@@ -2367,6 +2474,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query (dim_date): each Date.ToText([date_key], [Format = "MMM", Culture = "da-DK"])</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2431,6 +2543,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query (dim_date): each Date.ToText([date_key], [Format = "yyyy-MM"])</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2507,6 +2624,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query (dim_date): each Date.StartOfMonth([date_key])</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2575,6 +2697,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query (dim_date): each Date.WeekOfYear([date_key], Day.Monday)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2645,6 +2772,11 @@
       <c r="V20" t="inlineStr">
         <is>
           <t>Excel</t>
+        </is>
+      </c>
+      <c r="W20" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query (dim_date): each Date.DayOfWeek([date_key], Day.Monday) + 1</t>
         </is>
       </c>
     </row>
@@ -2711,6 +2843,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W21" t="inlineStr">
+        <is>
+          <t>Beregnet i Power Query (dim_date): each Date.ToText([date_key], [Format = "ddd", Culture = "da-DK"])</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2791,6 +2928,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W22" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_start_dt + silver.crm_prd_info.prd_key (afledt: row_number() over (order by pn.prd_start_dt, pn.prd_key)) ← bronze.crm_prd_info.prd_start_dt + bronze.crm_prd_info.prd_key (afledt: prd_start_dt::date; substring(prd_key from 7))</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2865,6 +3007,11 @@
       <c r="V23" t="inlineStr">
         <is>
           <t>Excel</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_id ← bronze.crm_prd_info.prd_id</t>
         </is>
       </c>
     </row>
@@ -2935,6 +3082,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_key ← bronze.crm_prd_info.prd_key (afledt: substring(prd_key from 7))</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3011,6 +3163,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_nm ← bronze.crm_prd_info.prd_nm</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3081,6 +3238,11 @@
       <c r="V26" t="inlineStr">
         <is>
           <t>Excel</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.cat_id ← bronze.crm_prd_info.prd_key (afledt: replace(substring(prd_key from 1 for 5), '-', '_'))</t>
         </is>
       </c>
     </row>
@@ -3159,6 +3321,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>silver.erp_px_cat_g1v2.cat ← bronze.erp_px_cat_g1v2.cat</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3231,6 +3398,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>silver.erp_px_cat_g1v2.subcat ← bronze.erp_px_cat_g1v2.subcat</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3299,6 +3471,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>silver.erp_px_cat_g1v2.maintenance ← bronze.erp_px_cat_g1v2.maintenance</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3373,6 +3550,11 @@
       <c r="V30" t="inlineStr">
         <is>
           <t>Excel</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_cost ← bronze.crm_prd_info.prd_cost (afledt: coalesce(prd_cost, 0))</t>
         </is>
       </c>
     </row>
@@ -3443,6 +3625,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_line ← bronze.crm_prd_info.prd_line (afledt: case when upper(trim(prd_line)) = 'M' then 'Mountain' when upper(trim(prd_line)…)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3513,6 +3700,11 @@
       <c r="V32" t="inlineStr">
         <is>
           <t>Excel</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>silver.crm_prd_info.prd_start_dt ← bronze.crm_prd_info.prd_start_dt (afledt: prd_start_dt::date)</t>
         </is>
       </c>
     </row>
@@ -3595,6 +3787,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W33" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_ord_num ← bronze.crm_sales_details.sls_ord_num</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3671,6 +3868,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>gold.dim_products.product_key ← silver.crm_prd_info.prd_start_dt + silver.crm_prd_info.prd_key (afledt: row_number() over (order by pn.prd_start_dt, pn.prd_key)) ← bronze.crm_prd_info.prd_start_dt + bronze.crm_prd_info.prd_key (afledt: prd_start_dt::date; substring(prd_key from 7))</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3751,6 +3953,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>gold.dim_customers.customer_key ← silver.crm_cust_info.cst_id (afledt: row_number() over (order by ci.cst_id)) ← bronze.crm_cust_info.cst_id</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3829,6 +4036,11 @@
       <c r="V36" t="inlineStr">
         <is>
           <t>Excel</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_order_dt ← bronze.crm_sales_details.sls_order_dt (afledt: case when sls_order_dt = 0 or length(sls_order_dt::text) != 8 then null else sl…)</t>
         </is>
       </c>
     </row>
@@ -3903,6 +4115,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_ship_dt ← bronze.crm_sales_details.sls_ship_dt (afledt: case when sls_ship_dt = 0 or length(sls_ship_dt::text) != 8 then null else sls_…)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3975,6 +4192,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_due_dt ← bronze.crm_sales_details.sls_due_dt (afledt: case when sls_due_dt = 0 or length(sls_due_dt::text) != 8 then null else sls_du…)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4051,6 +4273,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_sales ← bronze.crm_sales_details.sls_sales + bronze.crm_sales_details.sls_quantity + bronze.crm_sales_details.sls_price (afledt: case when sls_sales is null or sls_sales &lt;= 0 or sls_sales != sls_quantity * ab…)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4127,6 +4354,11 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_quantity ← bronze.crm_sales_details.sls_quantity</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4199,9 +4431,14 @@
           <t>Excel</t>
         </is>
       </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>silver.crm_sales_details.sls_price ← bronze.crm_sales_details.sls_price + bronze.crm_sales_details.sls_sales + bronze.crm_sales_details.sls_quantity (afledt: case when sls_price is null or sls_price &lt;= 0 then sls_sales / nullif(sls_quant…)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V41"/>
+  <autoFilter ref="A1:W41"/>
   <dataValidations count="1">
     <dataValidation sqref="U2:U41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Mangler,AI-forslag,Fra model,Redigeret,Godkendt"</formula1>

</xml_diff>